<commit_message>
login after few time
</commit_message>
<xml_diff>
--- a/boc_tms/boc_transport_backup.xlsx
+++ b/boc_tms/boc_transport_backup.xlsx
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-13 14:33:49</t>
+          <t>2026-08-17 14:27:58</t>
         </is>
       </c>
     </row>
@@ -709,10 +709,10 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>6.982516060148153</v>
+        <v>6.986306263988407</v>
       </c>
       <c r="H5" t="n">
-        <v>79.76559229157557</v>
+        <v>79.76359158572289</v>
       </c>
     </row>
     <row r="6">
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>6.956511208115466</v>
+        <v>6.956935279525572</v>
       </c>
       <c r="H11" t="n">
-        <v>79.89548238997631</v>
+        <v>79.89940986844411</v>
       </c>
     </row>
     <row r="12">
@@ -1564,7 +1564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -1991,7 +1991,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -2000,33 +2000,33 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Nimal Fernando</t>
+          <t>Mahinda Fernando</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>WP CAB-4943</t>
+          <t>WP CAB-3471</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Van</t>
+          <t>Double Cab</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Document courier</t>
+          <t>Head Office</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -2049,18 +2049,18 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>Transport Officer (from request)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-08-16T12:07:21</t>
+          <t>2026-08-17T11:03:31</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -2069,33 +2069,33 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="E8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Nimal Fernando</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
         <v>4</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Ajith Bandara</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>7</v>
-      </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>WP CAB-1763</t>
+          <t>WP CAB-4943</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Car</t>
+          <t>Van</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Branch inspection visit</t>
+          <t>Document courier</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -2129,7 +2129,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -2143,41 +2143,41 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Priyantha Dias</t>
+          <t>Ajith Bandara</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>WP NB-3363</t>
+          <t>WP CAB-1763</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Bus</t>
+          <t>Car</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Kurunegala Branch</t>
+          <t>Kandy Regional Office</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Cash in transit</t>
+          <t>Branch inspection visit</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -2198,42 +2198,42 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sunil Wickramasinghe</t>
+          <t>Priyantha Dias</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>WP CAB-2013</t>
+          <t>WP NB-3363</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Lorry</t>
+          <t>Bus</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Equipment delivery</t>
+          <t>Cash in transit</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -2267,7 +2267,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -2276,46 +2276,46 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Priyantha Dias</t>
+          <t>Sunil Wickramasinghe</t>
         </is>
       </c>
       <c r="G11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>WP CAB-2013</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Lorry</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
         <v>7</v>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>WP CAB-1763</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Car</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>2</v>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Colombo Fort Branch</t>
+          <t>Kurunegala Branch</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Cash in transit</t>
+          <t>Equipment delivery</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -2336,11 +2336,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -2362,24 +2362,24 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>WP CAB-3961</t>
+          <t>WP CAB-1763</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Lorry</t>
+          <t>Car</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>IT Division - Head Office</t>
+          <t>Colombo Fort Branch</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2405,37 +2405,37 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mahinda Dias</t>
+          <t>Priyantha Dias</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>WP CAB-2542</t>
+          <t>WP CAB-3961</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>VIP transport</t>
+          <t>Cash in transit</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2474,11 +2474,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2492,11 +2492,11 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Mahinda Kumara</t>
+          <t>Mahinda Dias</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -2513,16 +2513,16 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Negombo Branch</t>
+          <t>IT Division - Head Office</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Cash in transit</t>
+          <t>VIP transport</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2543,7 +2543,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2552,20 +2552,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ruwan Silva</t>
+          <t>Mahinda Kumara</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -2582,16 +2582,16 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Kandy Regional Office</t>
+          <t>Negombo Branch</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Staff transport</t>
+          <t>Cash in transit</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2612,42 +2612,42 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Mahinda Dias</t>
+          <t>Ruwan Silva</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>WP NB-3363</t>
+          <t>WP CAB-2542</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Bus</t>
+          <t>Lorry</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Document courier</t>
+          <t>Staff transport</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2681,55 +2681,55 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Priyantha Gunawardena</t>
+          <t>Mahinda Dias</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>WP CAB-3028</t>
+          <t>WP NB-3363</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Lorry</t>
+          <t>Bus</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>IT Division - Head Office</t>
+          <t>Kandy Regional Office</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cash in transit</t>
+          <t>Document courier</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2750,11 +2750,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2768,19 +2768,19 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ajith Bandara</t>
+          <t>Priyantha Gunawardena</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>WP CAB-4517</t>
+          <t>WP CAB-3028</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2789,16 +2789,16 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Kurunegala Branch</t>
+          <t>IT Division - Head Office</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Document courier</t>
+          <t>Cash in transit</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2819,68 +2819,137 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Ajith Bandara</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>WP CAB-4517</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Lorry</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>7</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Kurunegala Branch</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Document courier</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-08-16T12:07:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
         <v>5</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E20" t="n">
         <v>2</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Mahinda Dias</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G20" t="n">
         <v>4</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>WP CAB-4943</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Van</t>
         </is>
       </c>
-      <c r="J19" t="n">
+      <c r="J20" t="n">
         <v>6</v>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Negombo Branch</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Branch inspection visit</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>2026-08-16T12:07:21</t>
         </is>
@@ -2897,7 +2966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2987,6 +3056,79 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>kandy_branch</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-17T11:02:54</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>19</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-17T11:03:31</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Kandy Regional Office</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Mahinda Fernando</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>WP CAB-3471</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
changed into default windows theme
</commit_message>
<xml_diff>
--- a/boc_tms/boc_transport_backup.xlsx
+++ b/boc_tms/boc_transport_backup.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-17 14:27:58</t>
+          <t>2026-08-25 11:37:44</t>
         </is>
       </c>
     </row>
@@ -709,10 +709,10 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>6.986306263988407</v>
+        <v>6.9837996941802</v>
       </c>
       <c r="H5" t="n">
-        <v>79.76359158572289</v>
+        <v>79.7662631098716</v>
       </c>
     </row>
     <row r="6">
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>6.956935279525572</v>
+        <v>6.957214881668775</v>
       </c>
       <c r="H11" t="n">
-        <v>79.89940986844411</v>
+        <v>79.90338204513624</v>
       </c>
     </row>
     <row r="12">

</xml_diff>